<commit_message>
Actualiza documentacion del Reto (2026-10-10)
</commit_message>
<xml_diff>
--- a/proyecto-reto/04-fabricacion/hojas-viajeras/OF-2026-AGV-002_hoja-viajera.xlsx
+++ b/proyecto-reto/04-fabricacion/hojas-viajeras/OF-2026-AGV-002_hoja-viajera.xlsx
@@ -436,7 +436,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:I17"/>
+  <dimension ref="A1:I19"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="6" customWidth="1" min="1" max="1"/>
@@ -504,7 +504,7 @@
       </c>
       <c r="E6" t="inlineStr">
         <is>
-          <t>2026-10-10</t>
+          <t>2026-10-08</t>
         </is>
       </c>
     </row>
@@ -591,8 +591,16 @@
           <t>Surtir tubular de acero cal. 18 y verificar lista de corte. Material: OC-2026-006 (Marsa)</t>
         </is>
       </c>
-      <c r="D10" s="5" t="inlineStr"/>
-      <c r="E10" s="5" t="inlineStr"/>
+      <c r="D10" s="5" t="inlineStr">
+        <is>
+          <t>Rodrigo Herrera</t>
+        </is>
+      </c>
+      <c r="E10" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-05</t>
+        </is>
+      </c>
       <c r="F10" s="5" t="inlineStr"/>
       <c r="G10" s="5" t="inlineStr"/>
       <c r="H10" s="5" t="inlineStr"/>
@@ -612,7 +620,11 @@
           <t>Corte de tramos a medida y desbarbe de extremos</t>
         </is>
       </c>
-      <c r="D11" s="5" t="inlineStr"/>
+      <c r="D11" s="5" t="inlineStr">
+        <is>
+          <t>Rodrigo Herrera</t>
+        </is>
+      </c>
       <c r="E11" s="5" t="inlineStr"/>
       <c r="F11" s="5" t="inlineStr"/>
       <c r="G11" s="5" t="inlineStr"/>
@@ -633,7 +645,11 @@
           <t>Punteo, verificacion de escuadra y soldadura del bastidor</t>
         </is>
       </c>
-      <c r="D12" s="5" t="inlineStr"/>
+      <c r="D12" s="5" t="inlineStr">
+        <is>
+          <t>Rodrigo Herrera</t>
+        </is>
+      </c>
       <c r="E12" s="5" t="inlineStr"/>
       <c r="F12" s="5" t="inlineStr"/>
       <c r="G12" s="5" t="inlineStr"/>
@@ -654,9 +670,17 @@
           <t>Limpieza y esmerilado de cordones</t>
         </is>
       </c>
-      <c r="D13" s="5" t="inlineStr"/>
+      <c r="D13" s="5" t="inlineStr">
+        <is>
+          <t>Rodrigo Herrera</t>
+        </is>
+      </c>
       <c r="E13" s="5" t="inlineStr"/>
-      <c r="F13" s="5" t="inlineStr"/>
+      <c r="F13" s="5" t="inlineStr">
+        <is>
+          <t>2026-10-08</t>
+        </is>
+      </c>
       <c r="G13" s="5" t="inlineStr"/>
       <c r="H13" s="5" t="inlineStr"/>
       <c r="I13" s="5" t="inlineStr"/>
@@ -675,7 +699,11 @@
           <t>Escuadra, diagonales y planitud del bastidor</t>
         </is>
       </c>
-      <c r="D14" s="5" t="inlineStr"/>
+      <c r="D14" s="5" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
       <c r="E14" s="5" t="inlineStr"/>
       <c r="F14" s="5" t="inlineStr"/>
       <c r="G14" s="5" t="inlineStr"/>
@@ -696,13 +724,18 @@
           <t>Firma de calidad y entrega al subensamble mecanico del AGV</t>
         </is>
       </c>
-      <c r="D15" s="5" t="inlineStr"/>
+      <c r="D15" s="5" t="inlineStr">
+        <is>
+          <t>PENDIENTE</t>
+        </is>
+      </c>
       <c r="E15" s="5" t="inlineStr"/>
       <c r="F15" s="5" t="inlineStr"/>
       <c r="G15" s="5" t="inlineStr"/>
       <c r="H15" s="5" t="inlineStr"/>
       <c r="I15" s="5" t="inlineStr"/>
     </row>
+    <row r="16"/>
     <row r="17">
       <c r="A17" s="3" t="inlineStr">
         <is>
@@ -711,10 +744,12 @@
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>Registro posterior: fabricado la semana del 2026-10-05 al 2026-10-10 (fechas aproximadas). Subensamble de OF-2026-AGV-001.</t>
-        </is>
-      </c>
-    </row>
+          <t>Cortado y soldado por Rodrigo del 2026-10-05 al 2026-10-08 (confirmado 2026-10-10). Material: OC-2026-006 (Marsa). Subensamble de OF-2026-AGV-001. PENDIENTE: inspeccion dimensional (op 50), conteo de buenas/scrap y firma de calidad.</t>
+        </is>
+      </c>
+    </row>
+    <row r="18"/>
+    <row r="19"/>
   </sheetData>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>